<commit_message>
Loading OECD trade data
</commit_message>
<xml_diff>
--- a/paper 3/data/OECD trade facilitation A7 import export procedures.xlsx
+++ b/paper 3/data/OECD trade facilitation A7 import export procedures.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pliki\doktorat\ODDEA\WP1 digitalisation indexes comparison\ODDEA_index_analysis\paper 3\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD60354-12A8-468A-BC38-27D29B43601F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Table" sheetId="1" r:id="rId4"/>
-    <sheet name="Metadata" sheetId="2" r:id="rId5"/>
+    <sheet name="Table" sheetId="1" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="173">
-  <si>
-    <t>A7 - Import/export procedures - Performance</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
   <si>
     <t>Country</t>
   </si>
@@ -517,82 +519,88 @@
   </si>
   <si>
     <t>Zimbabwe</t>
-  </si>
-  <si>
-    <t>Data obtained from new-display.compareyourcountry.org in 2026-06-04 06:44:15 GMT</t>
   </si>
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <b val="true"/>
-        <i val="false"/>
-        <strike val="false"/>
-        <color rgb="FF000000"/>
-        <sz val="11"/>
-        <u val="none"/>
+        <family val="2"/>
+        <charset val="238"/>
       </rPr>
-      <t xml:space="preserve">A7 - Import/export procedures - Performance</t>
+      <t>A7 - Import/export procedures - Performance</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <b val="true"/>
-        <i val="false"/>
-        <strike val="false"/>
-        <color rgb="FF000000"/>
-        <sz val="11"/>
-        <u val="none"/>
+        <family val="2"/>
+        <charset val="238"/>
       </rPr>
-      <t xml:space="preserve">Data source</t>
+      <t>Data source</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Calibri"/>
-        <b val="false"/>
-        <i val="false"/>
-        <strike val="false"/>
-        <color rgb="ff0000ff"/>
-        <sz val="11"/>
-        <u val="single"/>
+        <family val="2"/>
+        <charset val="238"/>
       </rPr>
-      <t xml:space="preserve">Trade Facilitation Indicators Website</t>
+      <t>Trade Facilitation Indicators Website</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <b val="true"/>
-        <i val="false"/>
-        <strike val="false"/>
-        <color rgb="FF000000"/>
-        <sz val="11"/>
-        <u val="none"/>
+        <family val="2"/>
+        <charset val="238"/>
       </rPr>
-      <t xml:space="preserve">Indicator definition</t>
+      <t>Indicator definition</t>
     </r>
   </si>
-  <si/>
+  <si>
+    <t/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -600,31 +608,41 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -914,42 +932,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:E169"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D165"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.421387" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="5.855713" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="5.855713" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="5.855713" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="9.10" bestFit="true" style="0"/>
+    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="B1">
+        <v>2017</v>
+      </c>
+      <c r="C1">
+        <v>2019</v>
+      </c>
+      <c r="D1">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>2017</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>2019</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -961,9 +997,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -975,9 +1011,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -989,23 +1025,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -1017,12 +1053,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -1031,37 +1067,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1073,23 +1109,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1098,40 +1134,40 @@
         <v>1</v>
       </c>
       <c r="D14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1143,26 +1179,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1171,9 +1207,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1185,12 +1221,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1199,23 +1235,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -1224,40 +1260,40 @@
         <v>1</v>
       </c>
       <c r="D23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -1266,54 +1302,54 @@
         <v>1</v>
       </c>
       <c r="D26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -1325,82 +1361,82 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -1409,12 +1445,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -1423,65 +1459,65 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -1493,23 +1529,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44">
         <v>2</v>
@@ -1521,12 +1557,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45">
         <v>2</v>
@@ -1535,23 +1571,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B46">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C46">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D46">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B47">
         <v>2</v>
@@ -1563,65 +1599,65 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C48">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B51">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C51">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B52">
         <v>1</v>
@@ -1633,9 +1669,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B53">
         <v>2</v>
@@ -1647,135 +1683,135 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D56">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B57">
         <v>1</v>
       </c>
       <c r="C57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C59">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D59">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B60">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C60">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D60">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B61">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C61">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B62">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C62">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B63">
         <v>2</v>
@@ -1787,37 +1823,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64">
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B65">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B66">
         <v>1</v>
@@ -1829,23 +1865,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D67">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B68">
         <v>1</v>
@@ -1857,12 +1893,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>67</v>
-      </c>
-      <c r="B69">
-        <v>2</v>
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>69</v>
       </c>
       <c r="C69">
         <v>2</v>
@@ -1871,26 +1907,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D70">
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>69</v>
-      </c>
-      <c r="B71" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="B71">
+        <v>2</v>
       </c>
       <c r="C71">
         <v>2</v>
@@ -1899,9 +1935,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B72">
         <v>2</v>
@@ -1913,9 +1949,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B73">
         <v>2</v>
@@ -1927,9 +1963,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B74">
         <v>2</v>
@@ -1941,23 +1977,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D75">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B76">
         <v>2</v>
@@ -1969,9 +2005,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B77">
         <v>1</v>
@@ -1983,51 +2019,51 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78">
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D79">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B80">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C80">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D80">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B81">
         <v>2</v>
@@ -2039,96 +2075,96 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D82">
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D83">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D85">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D86">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B87">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C87">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D87">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B88">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C88">
         <v>1</v>
@@ -2137,51 +2173,51 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B89">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C89">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D89">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B90">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C90">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D90">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B91">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C91">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D91">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B92">
         <v>2</v>
@@ -2193,9 +2229,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B93">
         <v>1</v>
@@ -2204,26 +2240,26 @@
         <v>1</v>
       </c>
       <c r="D93">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B94">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C94">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D94">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B95">
         <v>1</v>
@@ -2232,40 +2268,40 @@
         <v>1</v>
       </c>
       <c r="D95">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B97">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C97">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D97">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B98">
         <v>2</v>
@@ -2277,40 +2313,40 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B99">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C99">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D99">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B100">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C100">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D100">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C101">
         <v>1</v>
@@ -2319,9 +2355,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B102">
         <v>1</v>
@@ -2333,9 +2369,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B103">
         <v>1</v>
@@ -2347,9 +2383,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B104">
         <v>1</v>
@@ -2361,9 +2397,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B105">
         <v>1</v>
@@ -2375,9 +2411,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B106">
         <v>1</v>
@@ -2389,9 +2425,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B107">
         <v>1</v>
@@ -2403,79 +2439,79 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B108">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C108">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D108">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D109">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B110">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C110">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D110">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B111">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C111">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D111">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B112">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C112">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D112">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B113">
         <v>1</v>
@@ -2487,9 +2523,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B114">
         <v>2</v>
@@ -2501,68 +2537,68 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B115">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C115">
         <v>1</v>
       </c>
       <c r="D115">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B116">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C116">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D116">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B117">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C117">
         <v>1</v>
       </c>
       <c r="D117">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B118">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C118">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D118">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B119">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C119">
         <v>1</v>
@@ -2571,9 +2607,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B120">
         <v>2</v>
@@ -2585,37 +2621,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B121">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C121">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D121">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B122">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C122">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D122">
         <v>2</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B123">
         <v>2</v>
@@ -2627,37 +2663,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B124">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C124">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D124">
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B125">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C125">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D125">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B126">
         <v>2</v>
@@ -2669,23 +2705,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B127">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C127">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D127">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B128">
         <v>2</v>
@@ -2697,79 +2733,79 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B129">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C129">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D129">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B130">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C130">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D130">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B131">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C131">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D131">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B132">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C132">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D132">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="133" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B133">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C133">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D133">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="134" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B134">
         <v>2</v>
@@ -2781,26 +2817,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B135">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C135">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D135">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B136">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C136">
         <v>2</v>
@@ -2809,26 +2845,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B137">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C137">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D137">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="138" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B138">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C138">
         <v>2</v>
@@ -2837,135 +2873,135 @@
         <v>2</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B139">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C139">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D139">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="140" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B140">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C140">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D140">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="141" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B141">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C141">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D141">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="142" spans="1:5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D142">
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B143">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C143">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="144" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B144">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C144">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D144">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="145" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B145">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C145">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D145">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="146" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B146">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C146">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D146">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="147" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B147">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C147">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D147">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="148" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B148">
         <v>1</v>
@@ -2977,9 +3013,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B149">
         <v>2</v>
@@ -2991,37 +3027,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B150">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C150">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D150">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="151" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B151">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C151">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D151">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="152" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B152">
         <v>2</v>
@@ -3033,9 +3069,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B153">
         <v>1</v>
@@ -3047,23 +3083,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B154">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C154">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D154">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="155" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B155">
         <v>1</v>
@@ -3075,37 +3111,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B156">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C156">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D156">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="157" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B157">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C157">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D157">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="158" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B158">
         <v>2</v>
@@ -3117,23 +3153,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B159">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C159">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D159">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B160">
         <v>2</v>
@@ -3145,9 +3181,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B161">
         <v>1</v>
@@ -3159,9 +3195,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B162">
         <v>2</v>
@@ -3173,9 +3209,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B163">
         <v>1</v>
@@ -3187,9 +3223,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B164">
         <v>2</v>
@@ -3201,9 +3237,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B165">
         <v>1</v>
@@ -3215,163 +3251,55 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
-      <c r="A166" t="s">
-        <v>165</v>
-      </c>
-      <c r="B166">
-        <v>2</v>
-      </c>
-      <c r="C166">
-        <v>2</v>
-      </c>
-      <c r="D166">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="167" spans="1:5">
-      <c r="A167" t="s">
-        <v>166</v>
-      </c>
-      <c r="B167">
-        <v>1</v>
-      </c>
-      <c r="C167">
-        <v>1</v>
-      </c>
-      <c r="D167">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="169" spans="1:5">
-      <c r="A169" t="s">
-        <v>167</v>
-      </c>
-    </row>
   </sheetData>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <mergeCells>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A169:H169"/>
-  </mergeCells>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.708252" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="80" customWidth="true" style="0"/>
-    <col min="3" max="3" width="80" customWidth="true" style="0"/>
+    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="true"/>
-              <i val="false"/>
-              <strike val="false"/>
-              <color rgb="FF000000"/>
-              <sz val="11"/>
-              <u val="none"/>
-            </rPr>
-            <t xml:space="preserve">A7 - Import/export procedures - Performance</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="true"/>
-              <i val="false"/>
-              <strike val="false"/>
-              <color rgb="FF000000"/>
-              <sz val="11"/>
-              <u val="none"/>
-            </rPr>
-            <t xml:space="preserve">Data source</t>
-          </r>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="false"/>
-              <i val="false"/>
-              <strike val="false"/>
-              <color rgb="ff0000ff"/>
-              <sz val="11"/>
-              <u val="single"/>
-            </rPr>
-            <t xml:space="preserve">Trade Facilitation Indicators Website</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="true"/>
-              <i val="false"/>
-              <strike val="false"/>
-              <color rgb="FF000000"/>
-              <sz val="11"/>
-              <u val="none"/>
-            </rPr>
-            <t xml:space="preserve">Indicator definition</t>
-          </r>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is/>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <mergeCells>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId_hyperlink_1"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>